<commit_message>
Update daily and weekly competitor tracking workbooks
</commit_message>
<xml_diff>
--- a/Broga_Competitor_Sales_Analysis.xlsx
+++ b/Broga_Competitor_Sales_Analysis.xlsx
@@ -12,8 +12,74 @@
 </workbook>
 </file>
 
+<file path=xl/comments2.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>Author</author>
+  </authors>
+  <commentList>
+    <comment ref="F50" authorId="0">
+      <text>
+        <r>
+          <t>Total units increased from 99 to 113 compared with 06/10/2025. Review whether this reflects a newly released unit scope.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="F222" authorId="0">
+      <text>
+        <r>
+          <t>Total units increased from 189 to 308 compared with 27/02/2026. Review whether this reflects a newly released unit scope.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="F225" authorId="0">
+      <text>
+        <r>
+          <t>Total units increased from 189 to 308 compared with 27/02/2026. Review whether this reflects a newly released unit scope.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="F227" authorId="0">
+      <text>
+        <r>
+          <t>Total units increased from 189 to 308 compared with 27/02/2026. Review whether this reflects a newly released unit scope.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="F229" authorId="0">
+      <text>
+        <r>
+          <t>Total units increased from 189 to 308 compared with 27/02/2026. Review whether this reflects a newly released unit scope.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="F231" authorId="0">
+      <text>
+        <r>
+          <t>Total units increased from 189 to 308 compared with 27/02/2026. Review whether this reflects a newly released unit scope.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="F233" authorId="0">
+      <text>
+        <r>
+          <t>Total units increased from 189 to 308 compared with 27/02/2026. Review whether this reflects a newly released unit scope.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="F235" authorId="0">
+      <text>
+        <r>
+          <t>Total units increased from 189 to 308 compared with 27/02/2026. Review whether this reflects a newly released unit scope.</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1781" uniqueCount="259">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1781" uniqueCount="258">
   <si>
     <t>BROGA COMPETITOR SALES ANALYSIS</t>
   </si>
@@ -705,9 +771,6 @@
     <t>45/136 signed</t>
   </si>
   <si>
-    <t>Earlier release scope (189 units)</t>
-  </si>
-  <si>
     <t>25% Signed (81/189 units)</t>
   </si>
   <si>
@@ -783,7 +846,7 @@
     <t>Scope</t>
   </si>
   <si>
-    <t>Birchpark remains four terrace groups and excludes rumah bandar. Sapphire uses the terrace-only comparison scope. Springvale keeps the 27-unit front-kitchen and 308-unit rear-kitchen groups separate.</t>
+    <t>Birchpark remains four terrace groups and excludes rumah bandar. Sapphire uses the terrace-only comparison scope. Springvale Group A remains 27 units. Group B is one continuing historical series: earlier records used 189 total units before the release scope increased to 308; the change is highlighted for review, not split into a new group.</t>
   </si>
   <si>
     <t>OneDrive destination</t>
@@ -796,7 +859,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -835,8 +898,12 @@
       <b/>
       <color rgb="FFB54708"/>
     </font>
+    <font>
+      <b/>
+      <color rgb="FF8A4B08"/>
+    </font>
   </fonts>
-  <fills count="9">
+  <fills count="10">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -878,6 +945,11 @@
         <fgColor rgb="FFFFF1D6"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFE4B5"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="3">
     <border>
@@ -909,7 +981,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -952,6 +1024,9 @@
     </xf>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -3590,7 +3665,7 @@
       <c r="E50" s="12">
         <v>70</v>
       </c>
-      <c r="F50" s="12">
+      <c r="F50" s="16">
         <v>113</v>
       </c>
       <c r="G50" s="15">
@@ -8280,7 +8355,7 @@
         <v>15</v>
       </c>
       <c r="C212" s="13" t="s">
-        <v>230</v>
+        <v>35</v>
       </c>
       <c r="D212" s="12" t="s">
         <v>121</v>
@@ -8295,7 +8370,7 @@
         <v>0.42857142857142855</v>
       </c>
       <c r="H212" s="13" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="I212" s="12" t="s">
         <v>117</v>
@@ -8324,7 +8399,7 @@
         <v>0.037037037037037035</v>
       </c>
       <c r="H213" s="13" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="I213" s="12" t="s">
         <v>117</v>
@@ -8338,7 +8413,7 @@
         <v>15</v>
       </c>
       <c r="C214" s="13" t="s">
-        <v>230</v>
+        <v>35</v>
       </c>
       <c r="D214" s="12" t="s">
         <v>121</v>
@@ -8353,7 +8428,7 @@
         <v>0.4444444444444444</v>
       </c>
       <c r="H214" s="13" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="I214" s="12" t="s">
         <v>117</v>
@@ -8382,7 +8457,7 @@
         <v>0</v>
       </c>
       <c r="H215" s="13" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="I215" s="12" t="s">
         <v>117</v>
@@ -8396,7 +8471,7 @@
         <v>15</v>
       </c>
       <c r="C216" s="13" t="s">
-        <v>230</v>
+        <v>35</v>
       </c>
       <c r="D216" s="12" t="s">
         <v>121</v>
@@ -8411,7 +8486,7 @@
         <v>0.656084656084656</v>
       </c>
       <c r="H216" s="13" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="I216" s="12" t="s">
         <v>117</v>
@@ -8440,7 +8515,7 @@
         <v>0</v>
       </c>
       <c r="H217" s="13" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="I217" s="12" t="s">
         <v>117</v>
@@ -8454,7 +8529,7 @@
         <v>15</v>
       </c>
       <c r="C218" s="13" t="s">
-        <v>230</v>
+        <v>35</v>
       </c>
       <c r="D218" s="12" t="s">
         <v>121</v>
@@ -8469,7 +8544,7 @@
         <v>0.783068783068783</v>
       </c>
       <c r="H218" s="13" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="I218" s="12" t="s">
         <v>117</v>
@@ -8498,7 +8573,7 @@
         <v>0.037037037037037035</v>
       </c>
       <c r="H219" s="13" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="I219" s="12" t="s">
         <v>117</v>
@@ -8512,7 +8587,7 @@
         <v>15</v>
       </c>
       <c r="C220" s="13" t="s">
-        <v>230</v>
+        <v>35</v>
       </c>
       <c r="D220" s="12" t="s">
         <v>121</v>
@@ -8527,7 +8602,7 @@
         <v>0.8148148148148148</v>
       </c>
       <c r="H220" s="13" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="I220" s="12" t="s">
         <v>117</v>
@@ -8556,7 +8631,7 @@
         <v>0.037037037037037035</v>
       </c>
       <c r="H221" s="13" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="I221" s="12" t="s">
         <v>117</v>
@@ -8578,14 +8653,14 @@
       <c r="E222" s="12">
         <v>160</v>
       </c>
-      <c r="F222" s="12">
+      <c r="F222" s="16">
         <v>308</v>
       </c>
       <c r="G222" s="15">
         <v>0.5194805194805194</v>
       </c>
       <c r="H222" s="13" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="I222" s="12" t="s">
         <v>117</v>
@@ -8614,7 +8689,7 @@
         <v>0.037037037037037035</v>
       </c>
       <c r="H223" s="13" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="I223" s="12" t="s">
         <v>117</v>
@@ -8643,7 +8718,7 @@
         <v>0.037037037037037035</v>
       </c>
       <c r="H224" s="13" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="I224" s="12" t="s">
         <v>128</v>
@@ -8665,14 +8740,14 @@
       <c r="E225" s="12">
         <v>161</v>
       </c>
-      <c r="F225" s="12">
+      <c r="F225" s="16">
         <v>308</v>
       </c>
       <c r="G225" s="15">
         <v>0.5227272727272727</v>
       </c>
       <c r="H225" s="13" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="I225" s="12" t="s">
         <v>128</v>
@@ -8701,7 +8776,7 @@
         <v>0.037037037037037035</v>
       </c>
       <c r="H226" s="13" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="I226" s="12" t="s">
         <v>128</v>
@@ -8723,14 +8798,14 @@
       <c r="E227" s="12">
         <v>161</v>
       </c>
-      <c r="F227" s="12">
+      <c r="F227" s="16">
         <v>308</v>
       </c>
       <c r="G227" s="15">
         <v>0.5227272727272727</v>
       </c>
       <c r="H227" s="13" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="I227" s="12" t="s">
         <v>128</v>
@@ -8759,7 +8834,7 @@
         <v>0.037037037037037035</v>
       </c>
       <c r="H228" s="13" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="I228" s="12" t="s">
         <v>128</v>
@@ -8781,14 +8856,14 @@
       <c r="E229" s="12">
         <v>161</v>
       </c>
-      <c r="F229" s="12">
+      <c r="F229" s="16">
         <v>308</v>
       </c>
       <c r="G229" s="15">
         <v>0.5227272727272727</v>
       </c>
       <c r="H229" s="13" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="I229" s="12" t="s">
         <v>128</v>
@@ -8817,7 +8892,7 @@
         <v>0.037037037037037035</v>
       </c>
       <c r="H230" s="13" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="I230" s="12" t="s">
         <v>128</v>
@@ -8839,14 +8914,14 @@
       <c r="E231" s="12">
         <v>161</v>
       </c>
-      <c r="F231" s="12">
+      <c r="F231" s="16">
         <v>308</v>
       </c>
       <c r="G231" s="15">
         <v>0.5227272727272727</v>
       </c>
       <c r="H231" s="13" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="I231" s="12" t="s">
         <v>128</v>
@@ -8875,7 +8950,7 @@
         <v>0.037037037037037035</v>
       </c>
       <c r="H232" s="13" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="I232" s="12" t="s">
         <v>128</v>
@@ -8897,14 +8972,14 @@
       <c r="E233" s="12">
         <v>161</v>
       </c>
-      <c r="F233" s="12">
+      <c r="F233" s="16">
         <v>308</v>
       </c>
       <c r="G233" s="15">
         <v>0.5227272727272727</v>
       </c>
       <c r="H233" s="13" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="I233" s="12" t="s">
         <v>128</v>
@@ -8933,7 +9008,7 @@
         <v>0.037037037037037035</v>
       </c>
       <c r="H234" s="13" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="I234" s="12" t="s">
         <v>128</v>
@@ -8955,14 +9030,14 @@
       <c r="E235" s="12">
         <v>161</v>
       </c>
-      <c r="F235" s="12">
+      <c r="F235" s="16">
         <v>308</v>
       </c>
       <c r="G235" s="15">
         <v>0.5227272727272727</v>
       </c>
       <c r="H235" s="13" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="I235" s="12" t="s">
         <v>128</v>
@@ -8991,7 +9066,7 @@
         <v>0.06040268456375839</v>
       </c>
       <c r="H236" s="13" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="I236" s="12" t="s">
         <v>117</v>
@@ -9020,7 +9095,7 @@
         <v>0.14093959731543623</v>
       </c>
       <c r="H237" s="13" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="I237" s="12" t="s">
         <v>117</v>
@@ -9049,7 +9124,7 @@
         <v>0.15436241610738255</v>
       </c>
       <c r="H238" s="13" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="I238" s="12" t="s">
         <v>117</v>
@@ -9078,7 +9153,7 @@
         <v>0.2080536912751678</v>
       </c>
       <c r="H239" s="13" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="I239" s="12" t="s">
         <v>117</v>
@@ -9107,7 +9182,7 @@
         <v>0.22818791946308725</v>
       </c>
       <c r="H240" s="13" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="I240" s="12" t="s">
         <v>117</v>
@@ -9136,7 +9211,7 @@
         <v>0.22818791946308725</v>
       </c>
       <c r="H241" s="13" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="I241" s="12" t="s">
         <v>117</v>
@@ -9165,7 +9240,7 @@
         <v>0.22818791946308725</v>
       </c>
       <c r="H242" s="13" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="I242" s="12" t="s">
         <v>128</v>
@@ -9194,7 +9269,7 @@
         <v>0.22818791946308725</v>
       </c>
       <c r="H243" s="13" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="I243" s="12" t="s">
         <v>128</v>
@@ -9223,7 +9298,7 @@
         <v>0.22818791946308725</v>
       </c>
       <c r="H244" s="13" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="I244" s="12" t="s">
         <v>128</v>
@@ -9252,7 +9327,7 @@
         <v>0.22818791946308725</v>
       </c>
       <c r="H245" s="13" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="I245" s="12" t="s">
         <v>128</v>
@@ -9281,7 +9356,7 @@
         <v>0.22818791946308725</v>
       </c>
       <c r="H246" s="13" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="I246" s="12" t="s">
         <v>128</v>
@@ -9310,7 +9385,7 @@
         <v>0.22818791946308725</v>
       </c>
       <c r="H247" s="13" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="I247" s="12" t="s">
         <v>128</v>
@@ -9320,6 +9395,7 @@
   <autoFilter ref="A1:I247"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <legacyDrawing r:id="rId2"/>
 </worksheet>
 </file>
 
@@ -9333,59 +9409,59 @@
   </cols>
   <sheetData>
     <row r="1" ht="46" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1" s="16" t="s">
+      <c r="A1" s="17" t="s">
+        <v>246</v>
+      </c>
+      <c r="B1" s="18" t="s">
         <v>247</v>
       </c>
-      <c r="B1" s="17" t="s">
+    </row>
+    <row r="2" ht="46" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" s="17" t="s">
+        <v>85</v>
+      </c>
+      <c r="B2" s="18" t="s">
         <v>248</v>
       </c>
     </row>
-    <row r="2" ht="46" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" s="16" t="s">
-        <v>85</v>
-      </c>
-      <c r="B2" s="17" t="s">
+    <row r="3" ht="46" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" s="17" t="s">
         <v>249</v>
       </c>
-    </row>
-    <row r="3" ht="46" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" s="16" t="s">
+      <c r="B3" s="18" t="s">
         <v>250</v>
       </c>
-      <c r="B3" s="17" t="s">
+    </row>
+    <row r="4" ht="46" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" s="17" t="s">
         <v>251</v>
       </c>
-    </row>
-    <row r="4" ht="46" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" s="16" t="s">
+      <c r="B4" s="18" t="s">
         <v>252</v>
       </c>
-      <c r="B4" s="17" t="s">
+    </row>
+    <row r="5" ht="46" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" s="17" t="s">
+        <v>98</v>
+      </c>
+      <c r="B5" s="18" t="s">
         <v>253</v>
       </c>
     </row>
-    <row r="5" ht="46" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" s="16" t="s">
-        <v>98</v>
-      </c>
-      <c r="B5" s="17" t="s">
+    <row r="6" ht="46" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" s="17" t="s">
         <v>254</v>
       </c>
-    </row>
-    <row r="6" ht="46" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A6" s="16" t="s">
+      <c r="B6" s="18" t="s">
         <v>255</v>
       </c>
-      <c r="B6" s="17" t="s">
+    </row>
+    <row r="7" ht="46" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" s="17" t="s">
         <v>256</v>
       </c>
-    </row>
-    <row r="7" ht="46" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A7" s="16" t="s">
+      <c r="B7" s="18" t="s">
         <v>257</v>
-      </c>
-      <c r="B7" s="17" t="s">
-        <v>258</v>
       </c>
     </row>
   </sheetData>

</xml_diff>